<commit_message>
Improved UX on Simulation override and updated flow.md, Architecture.md files
</commit_message>
<xml_diff>
--- a/Results/Demo_Case/Model/Model_accuracy_summary.xlsx
+++ b/Results/Demo_Case/Model/Model_accuracy_summary.xlsx
@@ -508,16 +508,16 @@
         <v>1604</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2063</v>
+        <v>0.2146</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1603</v>
+        <v>0.1653</v>
       </c>
       <c r="I2" t="n">
-        <v>0.42</v>
+        <v>0.43</v>
       </c>
       <c r="J2" t="n">
-        <v>0.9978</v>
+        <v>0.9976</v>
       </c>
     </row>
     <row r="3">
@@ -548,16 +548,16 @@
         <v>1604</v>
       </c>
       <c r="G3" t="n">
-        <v>2.2859</v>
+        <v>2.2456</v>
       </c>
       <c r="H3" t="n">
-        <v>1.7638</v>
+        <v>1.713</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>1.94</v>
       </c>
       <c r="J3" t="n">
-        <v>0.9703000000000001</v>
+        <v>0.9711</v>
       </c>
     </row>
     <row r="4">
@@ -612,16 +612,16 @@
         <v>1604</v>
       </c>
       <c r="G5" t="n">
-        <v>22.3707</v>
+        <v>21.2994</v>
       </c>
       <c r="H5" t="n">
-        <v>15.1044</v>
+        <v>15.15</v>
       </c>
       <c r="I5" t="n">
         <v>0.39</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8207</v>
+        <v>0.8377</v>
       </c>
     </row>
     <row r="6">
@@ -652,16 +652,16 @@
         <v>1604</v>
       </c>
       <c r="G6" t="n">
-        <v>312.1842</v>
+        <v>340.8123</v>
       </c>
       <c r="H6" t="n">
-        <v>234.3259</v>
+        <v>242.8293</v>
       </c>
       <c r="I6" t="n">
-        <v>0.59</v>
+        <v>0.61</v>
       </c>
       <c r="J6" t="n">
-        <v>0.9423</v>
+        <v>0.9374</v>
       </c>
     </row>
     <row r="7">
@@ -692,16 +692,16 @@
         <v>1604</v>
       </c>
       <c r="G7" t="n">
-        <v>7.1084</v>
+        <v>7.1489</v>
       </c>
       <c r="H7" t="n">
-        <v>5.997</v>
+        <v>5.9846</v>
       </c>
       <c r="I7" t="n">
-        <v>2.88</v>
+        <v>2.87</v>
       </c>
       <c r="J7" t="n">
-        <v>0.907</v>
+        <v>0.9098000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -732,16 +732,16 @@
         <v>1604</v>
       </c>
       <c r="G8" t="n">
-        <v>1.4639</v>
+        <v>1.4585</v>
       </c>
       <c r="H8" t="n">
-        <v>1.1063</v>
+        <v>1.125</v>
       </c>
       <c r="I8" t="n">
-        <v>0.57</v>
+        <v>0.58</v>
       </c>
       <c r="J8" t="n">
-        <v>0.9527</v>
+        <v>0.955</v>
       </c>
     </row>
     <row r="9">
@@ -772,16 +772,16 @@
         <v>1604</v>
       </c>
       <c r="G9" t="n">
-        <v>3.6443</v>
+        <v>4.2873</v>
       </c>
       <c r="H9" t="n">
-        <v>2.7431</v>
+        <v>2.8747</v>
       </c>
       <c r="I9" t="n">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="J9" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.9023</v>
       </c>
     </row>
     <row r="10">
@@ -812,16 +812,16 @@
         <v>1604</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2567</v>
+        <v>0.2534</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1998</v>
+        <v>0.1995</v>
       </c>
       <c r="I10" t="n">
         <v>0.76</v>
       </c>
       <c r="J10" t="n">
-        <v>0.9188</v>
+        <v>0.9229000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -852,16 +852,16 @@
         <v>1604</v>
       </c>
       <c r="G11" t="n">
-        <v>5.0809</v>
+        <v>5.7365</v>
       </c>
       <c r="H11" t="n">
-        <v>4.0695</v>
+        <v>3.9855</v>
       </c>
       <c r="I11" t="n">
-        <v>1.66</v>
+        <v>1.62</v>
       </c>
       <c r="J11" t="n">
-        <v>0.7673</v>
+        <v>0.7006</v>
       </c>
     </row>
     <row r="12">
@@ -916,16 +916,16 @@
         <v>1604</v>
       </c>
       <c r="G13" t="n">
-        <v>1.7287</v>
+        <v>1.6806</v>
       </c>
       <c r="H13" t="n">
-        <v>1.36</v>
+        <v>1.3426</v>
       </c>
       <c r="I13" t="n">
-        <v>2.61</v>
+        <v>2.58</v>
       </c>
       <c r="J13" t="n">
-        <v>0.7295</v>
+        <v>0.7373</v>
       </c>
     </row>
     <row r="14">
@@ -956,16 +956,16 @@
         <v>1604</v>
       </c>
       <c r="G14" t="n">
-        <v>0.7502</v>
+        <v>0.7662</v>
       </c>
       <c r="H14" t="n">
-        <v>0.5913</v>
+        <v>0.6055</v>
       </c>
       <c r="I14" t="n">
-        <v>1.45</v>
+        <v>1.48</v>
       </c>
       <c r="J14" t="n">
-        <v>0.8809</v>
+        <v>0.8784999999999999</v>
       </c>
     </row>
     <row r="15">
@@ -996,16 +996,16 @@
         <v>1604</v>
       </c>
       <c r="G15" t="n">
-        <v>69.94589999999999</v>
+        <v>80.9819</v>
       </c>
       <c r="H15" t="n">
-        <v>41.4523</v>
+        <v>42.8835</v>
       </c>
       <c r="I15" t="n">
-        <v>0.43</v>
+        <v>0.45</v>
       </c>
       <c r="J15" t="n">
-        <v>0.9802999999999999</v>
+        <v>0.9745</v>
       </c>
     </row>
     <row r="16">
@@ -1036,16 +1036,16 @@
         <v>1604</v>
       </c>
       <c r="G16" t="n">
-        <v>0.6491</v>
+        <v>0.6572</v>
       </c>
       <c r="H16" t="n">
-        <v>0.5095</v>
+        <v>0.514</v>
       </c>
       <c r="I16" t="n">
-        <v>2.09</v>
+        <v>2.11</v>
       </c>
       <c r="J16" t="n">
-        <v>0.7228</v>
+        <v>0.707</v>
       </c>
     </row>
     <row r="17">
@@ -1076,16 +1076,16 @@
         <v>1604</v>
       </c>
       <c r="G17" t="n">
-        <v>2.1605</v>
+        <v>2.1038</v>
       </c>
       <c r="H17" t="n">
-        <v>1.7013</v>
+        <v>1.684</v>
       </c>
       <c r="I17" t="n">
-        <v>11.7</v>
+        <v>11.83</v>
       </c>
       <c r="J17" t="n">
-        <v>0.7766</v>
+        <v>0.7834</v>
       </c>
     </row>
     <row r="18">
@@ -1116,16 +1116,16 @@
         <v>1604</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1815</v>
+        <v>0.1914</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1306</v>
+        <v>0.1355</v>
       </c>
       <c r="I18" t="n">
-        <v>15.74</v>
+        <v>16.28</v>
       </c>
       <c r="J18" t="n">
-        <v>0.629</v>
+        <v>0.5767</v>
       </c>
     </row>
     <row r="19">
@@ -1156,16 +1156,16 @@
         <v>1604</v>
       </c>
       <c r="G19" t="n">
-        <v>1.1777</v>
+        <v>1.1644</v>
       </c>
       <c r="H19" t="n">
-        <v>0.8328</v>
+        <v>0.8496</v>
       </c>
       <c r="I19" t="n">
-        <v>0.89</v>
+        <v>0.91</v>
       </c>
       <c r="J19" t="n">
-        <v>0.9064</v>
+        <v>0.906</v>
       </c>
     </row>
   </sheetData>

</xml_diff>